<commit_message>
Auto commit from remote update tool - 2026-09-17 17:39:10
</commit_message>
<xml_diff>
--- a/app/static/QuizMind_Template.xlsx
+++ b/app/static/QuizMind_Template.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,12 +418,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -449,7 +437,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>My Neural Quiz</t>
+          <t>TOEIC &amp; JLPT Standard Quiz Sample</t>
         </is>
       </c>
     </row>
@@ -461,7 +449,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>This is a sample quiz imported from Excel.</t>
+          <t>Comprehensive template supporting standalone questions, reading passages, and listening groups.</t>
         </is>
       </c>
     </row>
@@ -473,31 +461,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Foreign Languages</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tags</t>
+          <t>Time_Limit</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JLPT, N1, Grammar</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Time_Limit</t>
+          <t>Tags</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>toeic, jlpt, reading, listening</t>
         </is>
       </c>
     </row>
@@ -512,46 +500,81 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Option_A</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Option_B</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Option_C</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Option_D</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Group_ID</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Group_Title</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Passage_Content</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Group_Audio</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Group_Image</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Group_Order</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Allow_Shuffle</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
         <is>
           <t>Explanation</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>AI Analysis</t>
         </is>
@@ -560,84 +583,377 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hệ mặt trời có bao nhiêu hành tinh?</t>
+          <t>The company recently announced that it will _______ a new branch in Tokyo next month.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>open</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>opened</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>opening</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>opens</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Sao Diêm Vương không còn được coi là hành tinh từ năm 2006.</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Phân tích chuyên sâu về hệ mặt trời...</t>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Sau will + dong tu nguyen the (V-bare). Dap an dung: open.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Quy tac thi tuong lai don voi will trong TOEIC Part 5.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ai là người phát triển thuyết tương đối?</t>
+          <t>雨が_______前に、早く家に帰りましょう。</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Isaac Newton</t>
+          <t>降る</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Albert Einstein</t>
+          <t>降った</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Nikola Tesla</t>
+          <t>降って</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Galileo Galilei</t>
+          <t>降らない</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Albert Einstein công bố thuyết tương đối hẹp vào năm 1905.</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Phân tích về vật lý hiện đại...</t>
+          <t>降る</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Cau truc V-tu dien + mae ni (truoc khi lam gi).</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Ngu phap N3 V-ru + mae ni.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>What is the main purpose of the email?</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>To announce a schedule change for the conference</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>To confirm a hotel reservation</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>To request feedback on a presentation</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>To invite employees to a party</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>To announce a schedule change for the conference</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Questions 3-4 refer to the following email.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>From: conference@globaltech.com
+To: all_staff@globaltech.com
+Subject: Annual Conference Schedule Update
+Dear Team,
+Please be advised that the Annual Tech Innovation Summit originally scheduled for Friday, October 24 has been moved to Monday, October 27 due to venue maintenance. All keynote sessions will remain as previously outlined. Please update your calendars accordingly.</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Doan email thong bao doi lich hoi nghi thuong nien do bao tri dia diem.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Doc luot cau dau tien de tim purpose cua email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Why was the summit rescheduled?</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Due to bad weather conditions</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Because of venue maintenance</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Keynote speakers were unavailable</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Budget constraints</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Because of venue maintenance</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Dong 2: due to venue maintenance -&gt; Chon B.</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Chi tiet nguyen nhan trong email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Where does the conversation most likely take place?</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>At an airport check-in counter</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>In a hotel lobby</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>At a train station</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Inside a rental car office</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>At an airport check-in counter</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Questions 5-6 refer to the following listening dialogue.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>[Transcript]
+M: Good morning. I would like to check in for flight 402 to Chicago.
+W: Certainly, sir. May I see your passport and boarding pass?
+M: Here they are. Can I request an aisle seat, please?</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://actions.google.com/sounds/v1/ambiences/airport_terminal.ogg</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Nguoi nam noi: check in for flight 402 -&gt; Tai quay check-in san bay.</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Listening clue: flight 402, boarding pass, aisle seat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>What does the man request?</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A window seat</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>An aisle seat</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>A meal upgrade</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A flight refund</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>An aisle seat</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Nguoi nam hoi: Can I request an aisle seat, please?</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Chi tiet yeu cau cua nguoi nam.</t>
         </is>
       </c>
     </row>

</xml_diff>